<commit_message>
docs: add more quantum generative model papers
</commit_message>
<xml_diff>
--- a/metadata/QGenerative.xlsx
+++ b/metadata/QGenerative.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rbad6b27d8f1041a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R61a2f93089644c83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -399,19 +399,19 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Quantum Diffusion Model for Quark and Gluon Jet Generation</x:v>
+        <x:v>Dynamic Quantum Generative Adversarial Network Based on Residual Connection</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>AAAI Symposium Series</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>Mariia Baidachna; Rey Guadarrama; Gopal Ramesh Dahale; Tom Magorsch; Isabel Pedraza; Konstantin T. Matchev; Katia Matcheva; Kyoungchul Kong; Sergei Gleyzer</x:v>
+        <x:v>Han Qi; Jinxin Guo; Abdullah Gani</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>https://doi.org/10.1609/aaaiss.v7i1.36901</x:v>
+        <x:v>https://doi.org/10.1109/MAI69289.2026.11543537</x:v>
       </x:c>
       <x:c r="F5" t="str">
         <x:v>QGenerative</x:v>
@@ -419,19 +419,19 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Quantum generative adversarial network for image generation</x:v>
+        <x:v>Quantum generative adversarial networks: a comprehensive survey of theories, applications, and challenges in the NISQ era</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C6" t="str">
         <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>Mohammadsaleh Pajuhanfard; Ziwen Pan; Victor S. Sheng</x:v>
+        <x:v>Han Qi; Yihan Xu; Hao Wang; Abdullah Gani; Lip Yee Por</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>https://doi.org/10.1007/s00371-025-03915-8</x:v>
+        <x:v>https://doi.org/10.1007/s11128-026-05186-1</x:v>
       </x:c>
       <x:c r="F6" t="str">
         <x:v>QGenerative</x:v>
@@ -439,19 +439,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Quantum adversarial generation of high-resolution images</x:v>
+        <x:v>Parameter-efficient Quantum Denoising Diffusion Probabilistic Models with temporal encoding</x:v>
       </x:c>
       <x:c r="B7" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Springer Nature</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>QuanGong Ma; ChaoLong Hao; NianWen Si; Geng Chen; Jiale Zhang; Dan Qu</x:v>
+        <x:v>Xuefen Zhang; Chuangtao Chen</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>https://doi.org/10.1140/epjqt/s40507-024-00304-3</x:v>
+        <x:v>https://doi.org/10.1016/j.future.2025.107981</x:v>
       </x:c>
       <x:c r="F7" t="str">
         <x:v>QGenerative</x:v>
@@ -459,19 +459,19 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Quantum generative adversarial networks with dual generators</x:v>
+        <x:v>Quantum Diffusion Model for Quark and Gluon Jet Generation</x:v>
       </x:c>
       <x:c r="B8" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>IOP Publishing</x:v>
+        <x:v>AAAI Symposium Series</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>Quangong Ma; Chaolong Hao; NianWen Si; Dan Qu</x:v>
+        <x:v>Mariia Baidachna; Rey Guadarrama; Gopal Ramesh Dahale; Tom Magorsch; Isabel Pedraza; Konstantin T. Matchev; Katia Matcheva; Kyoungchul Kong; Sergei Gleyzer</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>https://doi.org/10.1088/2632-2153/ae0bf7</x:v>
+        <x:v>https://doi.org/10.1609/aaaiss.v7i1.36901</x:v>
       </x:c>
       <x:c r="F8" t="str">
         <x:v>QGenerative</x:v>
@@ -479,19 +479,19 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Quantum generative adversarial network based on the quantum Born machine</x:v>
+        <x:v>Quantum generative adversarial network for image generation</x:v>
       </x:c>
       <x:c r="B9" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>Elsevier</x:v>
+        <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>Yifan Ding; Zi Li; Nanrun Zhou</x:v>
+        <x:v>Mohammadsaleh Pajuhanfard; Ziwen Pan; Victor S. Sheng</x:v>
       </x:c>
       <x:c r="E9" t="str">
-        <x:v>https://doi.org/10.1016/j.aei.2025.103622</x:v>
+        <x:v>https://doi.org/10.1007/s00371-025-03915-8</x:v>
       </x:c>
       <x:c r="F9" t="str">
         <x:v>QGenerative</x:v>
@@ -499,19 +499,19 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Quantum generative classification with mixed states</x:v>
+        <x:v>Quantum adversarial generation of high-resolution images</x:v>
       </x:c>
       <x:c r="B10" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>IOP Publishing</x:v>
+        <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>Diego H. Useche; Sergio Quiroga-Sandoval; Sebastian L. Molina; Vladimir Vargas-Calderón; Juan E. Ardila-García; Fabio A. González</x:v>
+        <x:v>QuanGong Ma; ChaoLong Hao; NianWen Si; Geng Chen; Jiale Zhang; Dan Qu</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>https://doi.org/10.1088/2058-9565/adf350</x:v>
+        <x:v>https://doi.org/10.1140/epjqt/s40507-024-00304-3</x:v>
       </x:c>
       <x:c r="F10" t="str">
         <x:v>QGenerative</x:v>
@@ -519,19 +519,19 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Quantum Diffusion Models for Few-Shot Learning</x:v>
+        <x:v>Quantum generative adversarial networks with dual generators</x:v>
       </x:c>
       <x:c r="B11" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>Springer Nature</x:v>
+        <x:v>IOP Publishing</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>Ruhan Wang; Ye Wang; Jing Liu; Toshiaki Koike-Akino</x:v>
+        <x:v>Quangong Ma; Chaolong Hao; NianWen Si; Dan Qu</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>https://doi.org/10.1007/978-3-032-15931-1</x:v>
+        <x:v>https://doi.org/10.1088/2632-2153/ae0bf7</x:v>
       </x:c>
       <x:c r="F11" t="str">
         <x:v>QGenerative</x:v>
@@ -539,19 +539,19 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>Quantum generative adversarial networks: Bridging classical and quantum realms</x:v>
+        <x:v>Quantum generative adversarial network based on the quantum Born machine</x:v>
       </x:c>
       <x:c r="B12" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>International Conference on Intelligent Systems, Metaheuristics &amp; Swarm Intelligence</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>Nokhwal, Sahil, et al.</x:v>
+        <x:v>Yifan Ding; Zi Li; Nanrun Zhou</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3665065.3665082</x:v>
+        <x:v>https://doi.org/10.1016/j.aei.2025.103622</x:v>
       </x:c>
       <x:c r="F12" t="str">
         <x:v>QGenerative</x:v>
@@ -559,20 +559,19 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>Quantum Generative Adversarial Networks: Generating and Detecting Quantum Product States
-</x:v>
+        <x:v>Quantum generative classification with mixed states</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>IOP Publishing</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>Steck, James E., and Elizabeth C. Behrman.</x:v>
+        <x:v>Diego H. Useche; Sergio Quiroga-Sandoval; Sebastian L. Molina; Vladimir Vargas-Calderón; Juan E. Ardila-García; Fabio A. González</x:v>
       </x:c>
       <x:c r="E13" t="str">
-        <x:v>https://arxiv.org/abs/2408.12620</x:v>
+        <x:v>https://doi.org/10.1088/2058-9565/adf350</x:v>
       </x:c>
       <x:c r="F13" t="str">
         <x:v>QGenerative</x:v>
@@ -580,20 +579,19 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>HQ-DCGAN: Hybrid quantum deep convolutional generative adversarial network approach for ECG generation
-</x:v>
+        <x:v>Quantum Diffusion Models for Few-Shot Learning</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>Knowledge-Based Systems</x:v>
+        <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="D14" t="str">
-        <x:v>Qu, Zhiguo, Weilong Chen, and Prayag Tiwari.</x:v>
+        <x:v>Ruhan Wang; Ye Wang; Jing Liu; Toshiaki Koike-Akino</x:v>
       </x:c>
       <x:c r="E14" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/pii/S0950705124008943</x:v>
+        <x:v>https://doi.org/10.1007/978-3-032-15931-1</x:v>
       </x:c>
       <x:c r="F14" t="str">
         <x:v>QGenerative</x:v>
@@ -601,19 +599,19 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>Carbon market risk estimation using quantum conditional generative adversarial network and amplitude estimation.</x:v>
+        <x:v>Generative quantum advantage for classical and quantum problems</x:v>
       </x:c>
       <x:c r="B15" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>Energy Conversion and Economics</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>Zhou, Xiyuan, et al.</x:v>
+        <x:v>Hsin-Yuan Huang; Michael Broughton; Norhan Eassa; Hartmut Neven; Ryan Babbush; Jarrod R. McClean</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>https://ietresearch.onlinelibrary.wiley.com/doi/full/10.1049/enc2.12122</x:v>
+        <x:v>https://arxiv.org/abs/2509.09033</x:v>
       </x:c>
       <x:c r="F15" t="str">
         <x:v>QGenerative</x:v>
@@ -621,19 +619,19 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Variational Quantum Circuits Enhanced Generative Adversarial Network</x:v>
+        <x:v>Parameterized quantum circuits as universal generative models for continuous multivariate distributions</x:v>
       </x:c>
       <x:c r="B16" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>Shu, Runqiu, et al.</x:v>
+        <x:v>Alice Barthe; Michele Grossi; Sofia Vallecorsa; Jordi Tura; Vedran Dunjko</x:v>
       </x:c>
       <x:c r="E16" t="str">
-        <x:v>https://arxiv.org/pdf/2402.01791</x:v>
+        <x:v>https://doi.org/10.1038/s41534-025-01064-3</x:v>
       </x:c>
       <x:c r="F16" t="str">
         <x:v>QGenerative</x:v>
@@ -641,19 +639,19 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>Hamiltonian quantum generative adversarial networks</x:v>
+        <x:v>Quantum Latent Diffusion Models</x:v>
       </x:c>
       <x:c r="B17" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>Physical Review Research </x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>Kim, Leeseok, Seth Lloyd, and Milad Marvian.</x:v>
+        <x:v>Francesca De Falco; Andrea Ceschini; Alessandro Sebastianelli; Bertrand Le Saux; Massimo Panella</x:v>
       </x:c>
       <x:c r="E17" t="str">
-        <x:v>https://journals.aps.org/prresearch/pdf/10.1103/PhysRevResearch.6.033019</x:v>
+        <x:v>https://arxiv.org/abs/2501.11174</x:v>
       </x:c>
       <x:c r="F17" t="str">
         <x:v>QGenerative</x:v>
@@ -661,20 +659,19 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>A Characterization of Quantum Generative Models
-</x:v>
+        <x:v>Denoising diffusion models with optimized quantum implicit neural networks for image generation</x:v>
       </x:c>
       <x:c r="B18" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>ACM Transactions on Quantum Computing</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>Riofrio, Carlos A., et al.</x:v>
+        <x:v>Jiale Zhang; Xilong Che; Yuzhe Fan; Shun Peng; Geng Chen; Quangong Ma; Juncheng Hu</x:v>
       </x:c>
       <x:c r="E18" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3655027</x:v>
+        <x:v>https://doi.org/10.1016/j.future.2025.107875</x:v>
       </x:c>
       <x:c r="F18" t="str">
         <x:v>QGenerative</x:v>
@@ -682,20 +679,19 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>Investigating the application of Quantum-Enhanced Generative
-Adversarial Networks in optimizing supply chain processes</x:v>
+        <x:v>Quantum generative adversarial networks: Bridging classical and quantum realms</x:v>
       </x:c>
       <x:c r="B19" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>Neurocomputing</x:v>
+        <x:v>International Conference on Intelligent Systems, Metaheuristics &amp; Swarm Intelligence</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>Pahune, Saurabh A., and Noopur Rewatkar.</x:v>
+        <x:v>Nokhwal, Sahil, et al.</x:v>
       </x:c>
       <x:c r="E19" t="str">
-        <x:v>https://www.researchgate.net/profile/Saurabh-Pahune-2/publication/380460708_Investigating_the_application_of_Quantum-Enhanced_Generative_Adversarial_Networks_in_optimizing_supply_chain_processes/links/663e498e352430415396d58a/Investigating-the-application-of-Quantum-Enhanced-Generative-Adversarial-Networks-in-optimizing-supply-chain-processes.pdf</x:v>
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3665065.3665082</x:v>
       </x:c>
       <x:c r="F19" t="str">
         <x:v>QGenerative</x:v>
@@ -716,7 +712,7 @@
         <x:v>Steck, James E., and Elizabeth C. Behrman.</x:v>
       </x:c>
       <x:c r="E20" t="str">
-        <x:v>https://www.techrxiv.org/doi/full/10.36227/techrxiv.172349428.83803592/v1</x:v>
+        <x:v>https://arxiv.org/abs/2408.12620</x:v>
       </x:c>
       <x:c r="F20" t="str">
         <x:v>QGenerative</x:v>
@@ -724,492 +720,496 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
+        <x:v>HQ-DCGAN: Hybrid quantum deep convolutional generative adversarial network approach for ECG generation
+</x:v>
+      </x:c>
+      <x:c r="B21" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Knowledge-Based Systems</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>Qu, Zhiguo, Weilong Chen, and Prayag Tiwari.</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/pii/S0950705124008943</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>Carbon market risk estimation using quantum conditional generative adversarial network and amplitude estimation.</x:v>
+      </x:c>
+      <x:c r="B22" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Energy Conversion and Economics</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Zhou, Xiyuan, et al.</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>https://ietresearch.onlinelibrary.wiley.com/doi/full/10.1049/enc2.12122</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>Variational Quantum Circuits Enhanced Generative Adversarial Network</x:v>
+      </x:c>
+      <x:c r="B23" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Shu, Runqiu, et al.</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>https://arxiv.org/pdf/2402.01791</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>Hamiltonian quantum generative adversarial networks</x:v>
+      </x:c>
+      <x:c r="B24" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Physical Review Research </x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>Kim, Leeseok, Seth Lloyd, and Milad Marvian.</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>https://journals.aps.org/prresearch/pdf/10.1103/PhysRevResearch.6.033019</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>A Characterization of Quantum Generative Models
+</x:v>
+      </x:c>
+      <x:c r="B25" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>ACM Transactions on Quantum Computing</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>Riofrio, Carlos A., et al.</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3655027</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>Investigating the application of Quantum-Enhanced Generative
+Adversarial Networks in optimizing supply chain processes</x:v>
+      </x:c>
+      <x:c r="B26" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Neurocomputing</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>Pahune, Saurabh A., and Noopur Rewatkar.</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>https://www.researchgate.net/profile/Saurabh-Pahune-2/publication/380460708_Investigating_the_application_of_Quantum-Enhanced_Generative_Adversarial_Networks_in_optimizing_supply_chain_processes/links/663e498e352430415396d58a/Investigating-the-application-of-Quantum-Enhanced-Generative-Adversarial-Networks-in-optimizing-supply-chain-processes.pdf</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>Quantum Generative Adversarial Networks: Generating and Detecting Quantum Product States
+</x:v>
+      </x:c>
+      <x:c r="B27" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Steck, James E., and Elizabeth C. Behrman.</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>https://www.techrxiv.org/doi/full/10.36227/techrxiv.172349428.83803592/v1</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
         <x:v>Photonic quantum generative adversarial networks for classical data
 </x:v>
       </x:c>
-      <x:c r="B21" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C21" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D21" t="str">
+      <x:c r="B28" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
         <x:v>Sedrakyan, Tigran, and Alexia Salavrakos.</x:v>
       </x:c>
-      <x:c r="E21" t="str">
+      <x:c r="E28" t="str">
         <x:v>https://arxiv.org/pdf/2405.06023</x:v>
       </x:c>
-      <x:c r="F21" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" t="str">
+      <x:c r="F28" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
         <x:v>A super resolution method based on generative adversarial networks with quantum feature enhancement: Application to aerial agricultural images
 </x:v>
       </x:c>
-      <x:c r="B22" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C22" t="str">
+      <x:c r="B29" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
         <x:v>Neurocomputing</x:v>
       </x:c>
-      <x:c r="D22" t="str">
+      <x:c r="D29" t="str">
         <x:v>Pu, Ziqiang, et al.</x:v>
       </x:c>
-      <x:c r="E22" t="str">
+      <x:c r="E29" t="str">
         <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0925231224001176</x:v>
       </x:c>
-      <x:c r="F22" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" t="str">
+      <x:c r="F29" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
         <x:v>Investigate the Performance of Distribution Loading with Conditional Quantum Generative Adversarial Network Algorithm on Quantum Hardware with Error Suppression
 </x:v>
       </x:c>
-      <x:c r="B23" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C23" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D23" t="str">
+      <x:c r="B30" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
         <x:v>Pham, Anh, and Andrew Vlasic.</x:v>
       </x:c>
-      <x:c r="E23" t="str">
+      <x:c r="E30" t="str">
         <x:v>https://arxiv.org/pdf/2406.09341</x:v>
       </x:c>
-      <x:c r="F23" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" t="str">
+      <x:c r="F30" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
         <x:v>Data augmentation experiments with style-based
 quantum generative adversarial networks on
 trapped-ion and superconducting-qubit technologies</x:v>
       </x:c>
-      <x:c r="B24" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C24" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D24" t="str">
+      <x:c r="B31" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
         <x:v>Baglio, Julien.</x:v>
       </x:c>
-      <x:c r="E24" t="str">
+      <x:c r="E31" t="str">
         <x:v>https://arxiv.org/pdf/2405.04401</x:v>
       </x:c>
-      <x:c r="F24" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" t="str">
+      <x:c r="F31" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
         <x:v>Design of Nanoscale Quantum Interconnects Aided by Conditional Generative Adversarial Networks
 </x:v>
       </x:c>
-      <x:c r="B25" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C25" t="str">
+      <x:c r="B32" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
         <x:v>Applied Sciences </x:v>
       </x:c>
-      <x:c r="D25" t="str">
+      <x:c r="D32" t="str">
         <x:v>Preda, Amanda Teodora, et al.</x:v>
       </x:c>
-      <x:c r="E25" t="str">
+      <x:c r="E32" t="str">
         <x:v>https://www.mdpi.com/2076-3417/14/3/1111</x:v>
       </x:c>
-      <x:c r="F25" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" t="str">
+      <x:c r="F32" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
         <x:v>Quantum generative adversarial networks based on a readout error mitigation method with fault tolerant mechanism</x:v>
       </x:c>
-      <x:c r="B26" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C26" t="str">
+      <x:c r="B33" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
         <x:v>Chinese Physics </x:v>
       </x:c>
-      <x:c r="D26" t="str">
+      <x:c r="D33" t="str">
         <x:v>Zhao, Run-Sheng, et al.</x:v>
       </x:c>
-      <x:c r="E26" t="str">
+      <x:c r="E33" t="str">
         <x:v>https://iopscience.iop.org/article/10.1088/1674-1056/ad02e7/meta</x:v>
       </x:c>
-      <x:c r="F26" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" t="str">
+      <x:c r="F33" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
         <x:v>A framework for demonstrating practical quantum advantage: comparing quantum against classical generative models
 </x:v>
       </x:c>
-      <x:c r="B27" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C27" t="str">
+      <x:c r="B34" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
         <x:v>Communications Physics </x:v>
       </x:c>
-      <x:c r="D27" t="str">
+      <x:c r="D34" t="str">
         <x:v>Hibat-Allah, Mohamed, et al.</x:v>
       </x:c>
-      <x:c r="E27" t="str">
+      <x:c r="E34" t="str">
         <x:v>https://www.nature.com/articles/s42005-024-01552-6</x:v>
       </x:c>
-      <x:c r="F27" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" t="str">
+      <x:c r="F34" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
         <x:v>Non-native Quantum Generative Optimization with Adversarial Autoencoders</x:v>
       </x:c>
-      <x:c r="B28" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C28" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D28" t="str">
+      <x:c r="B35" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
         <x:v>Wilson, Blake A., et al.</x:v>
       </x:c>
-      <x:c r="E28" t="str">
+      <x:c r="E35" t="str">
         <x:v>https://arxiv.org/pdf/2407.13830</x:v>
       </x:c>
-      <x:c r="F28" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" t="str">
+      <x:c r="F35" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
         <x:v>Radial Basis Function-based Quantum Hybrid Classical Generative Adversarial Networks for Enhanced Image Quality and Training Stability.</x:v>
       </x:c>
-      <x:c r="B29" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C29" t="str">
+      <x:c r="B36" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
         <x:v>PREPRINT (Version 1) available at Research Square</x:v>
       </x:c>
-      <x:c r="D29" t="str">
+      <x:c r="D36" t="str">
         <x:v>Xu, Zuyu, et al.</x:v>
       </x:c>
-      <x:c r="E29" t="str">
+      <x:c r="E36" t="str">
         <x:v>https://www.researchsquare.com/article/rs-4195599/v1</x:v>
       </x:c>
-      <x:c r="F29" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" t="str">
+      <x:c r="F36" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
         <x:v>A Hybrid Quantum-Classical AI-Based Detection Strategy for Generative Adversarial Network-Based Deepfake Attacks on an Autonomous Vehicle Traffic Sign Classification System.</x:v>
       </x:c>
-      <x:c r="B30" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C30" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D30" t="str">
+      <x:c r="B37" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
         <x:v>Salek, M. Sabbir, Shaozhi Li, and Mashrur Chowdhury.</x:v>
       </x:c>
-      <x:c r="E30" t="str">
+      <x:c r="E37" t="str">
         <x:v>https://arxiv.org/abs/2409.17311</x:v>
       </x:c>
-      <x:c r="F30" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" t="str">
+      <x:c r="F37" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
         <x:v>VAE-QWGAN: Improving Quantum GANs for High Resolution Image Generation
 </x:v>
       </x:c>
-      <x:c r="B31" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C31" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D31" t="str">
+      <x:c r="B38" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
         <x:v>Thomas, Aaron Mark, and Sharu Theresa Jose.</x:v>
       </x:c>
-      <x:c r="E31" t="str">
+      <x:c r="E38" t="str">
         <x:v>https://arxiv.org/pdf/2409.10339</x:v>
       </x:c>
-      <x:c r="F31" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" t="str">
+      <x:c r="F38" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
         <x:v>Quantum Generative Learning for High-Resolution Medical Image Generation
 </x:v>
       </x:c>
-      <x:c r="B32" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C32" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D32" t="str">
+      <x:c r="B39" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
         <x:v>Khatun, Amena, et al.</x:v>
       </x:c>
-      <x:c r="E32" t="str">
+      <x:c r="E39" t="str">
         <x:v>https://arxiv.org/abs/2406.13196</x:v>
       </x:c>
-      <x:c r="F32" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" t="str">
+      <x:c r="F39" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
         <x:v>Enhancing combinatorial optimization with classical and quantum generative models
 </x:v>
       </x:c>
-      <x:c r="B33" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C33" t="str">
+      <x:c r="B40" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
         <x:v>Nature Communications</x:v>
       </x:c>
-      <x:c r="D33" t="str">
+      <x:c r="D40" t="str">
         <x:v>Alcazar, Javier, et al.</x:v>
       </x:c>
-      <x:c r="E33" t="str">
+      <x:c r="E40" t="str">
         <x:v>https://www.nature.com/articles/s41467-024-46959-5</x:v>
       </x:c>
-      <x:c r="F33" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" t="str">
+      <x:c r="F40" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
         <x:v>Benchmarking Quantum Generative Learning: A Study on Scalability and Noise Resilience using QUARK
 </x:v>
       </x:c>
-      <x:c r="B34" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C34" t="str">
+      <x:c r="B41" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
         <x:v>KI-Künstliche Intelligenz</x:v>
       </x:c>
-      <x:c r="D34" t="str">
+      <x:c r="D41" t="str">
         <x:v>Kiwit, Florian J., et al.</x:v>
       </x:c>
-      <x:c r="E34" t="str">
+      <x:c r="E41" t="str">
         <x:v>https://link.springer.com/article/10.1007/s13218-024-00864-7</x:v>
       </x:c>
-      <x:c r="F34" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" t="str">
+      <x:c r="F41" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
         <x:v>Protocols for trainable and differentiable quantum generative modeling</x:v>
       </x:c>
-      <x:c r="B35" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C35" t="str">
+      <x:c r="B42" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
         <x:v>Physical Review Research </x:v>
       </x:c>
-      <x:c r="D35" t="str">
+      <x:c r="D42" t="str">
         <x:v>Kyriienko, Oleksandr, Annie E. Paine, and Vincent E. Elfving.</x:v>
       </x:c>
-      <x:c r="E35" t="str">
+      <x:c r="E42" t="str">
         <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.6.033291</x:v>
       </x:c>
-      <x:c r="F35" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" t="str">
+      <x:c r="F42" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
         <x:v>Exploring Biological Neuronal Correlations with Quantum Generative Models
 </x:v>
       </x:c>
-      <x:c r="B36" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C36" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D36" t="str">
+      <x:c r="B43" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
         <x:v>Hernandes, Vinicius, and Eliska Greplova.</x:v>
       </x:c>
-      <x:c r="E36" t="str">
+      <x:c r="E43" t="str">
         <x:v>https://arxiv.org/abs/2409.09125</x:v>
       </x:c>
-      <x:c r="F36" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" t="str">
+      <x:c r="F43" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
         <x:v>Generating Universal Adversarial Perturbations for Quantum Classifiers
 </x:v>
       </x:c>
-      <x:c r="B37" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C37" t="str">
+      <x:c r="B44" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
         <x:v>Proceedings of the AAAI Conference on Artificial Intelligence</x:v>
       </x:c>
-      <x:c r="D37" t="str">
+      <x:c r="D44" t="str">
         <x:v>Anil, Gautham, Vishnu Vinod, and Apurva Narayan.</x:v>
       </x:c>
-      <x:c r="E37" t="str">
+      <x:c r="E44" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/28963</x:v>
-      </x:c>
-      <x:c r="F37" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" t="str">
-        <x:v>Investigating Training Dynamics of Quantum Generative Adversarial Networks</x:v>
-      </x:c>
-      <x:c r="B38" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C38" t="str">
-        <x:v>Bulletin of the American Physical Society </x:v>
-      </x:c>
-      <x:c r="D38" t="str">
-        <x:v>Rajapakse, Renuka, and McCord Murray.</x:v>
-      </x:c>
-      <x:c r="E38" t="str">
-        <x:v>https://meetings.aps.org/Meeting/DAMOP24/Session/R11.1</x:v>
-      </x:c>
-      <x:c r="F38" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" t="str">
-        <x:v>Latent Style-based Quantum GAN for high-quality Image Generation</x:v>
-      </x:c>
-      <x:c r="B39" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C39" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D39" t="str">
-        <x:v>Chang, Su Yeon, et al.</x:v>
-      </x:c>
-      <x:c r="E39" t="str">
-        <x:v>https://arxiv.org/pdf/2406.02668</x:v>
-      </x:c>
-      <x:c r="F39" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" t="str">
-        <x:v>Recent Advances for Quantum Neural Networks in Generative Learning</x:v>
-      </x:c>
-      <x:c r="B40" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C40" t="str">
-        <x:v> IEEE Transactions on Pattern Analysis and Machine Intelligence</x:v>
-      </x:c>
-      <x:c r="D40" t="str">
-        <x:v>Jinkai Tian, Xiaoyu Sun, Yuxuan Du, Shanshan Zhao, Qing Liu, Kaining Zhang, Wei Yi, Wanrong Huang, Chaoyue Wang, Xingyao Wu, Min-Hsiu Hsieh, Tongliang Liu, Wenjing Yang, Dacheng Tao</x:v>
-      </x:c>
-      <x:c r="E40" t="str">
-        <x:v>https://doi.org/10.1109/TPAMI.2023.3272029</x:v>
-      </x:c>
-      <x:c r="F40" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" t="str">
-        <x:v>Hybrid quantum–classical generative adversarial networks for image generation via learning discrete distribution</x:v>
-      </x:c>
-      <x:c r="B41" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C41" t="str">
-        <x:v>ScienceDirect</x:v>
-      </x:c>
-      <x:c r="D41" t="str">
-        <x:v>Nan-Run Zhou,  Tian-Feng Zhang,  Xin-Wen Xie,  Jun-Yun Wu</x:v>
-      </x:c>
-      <x:c r="E41" t="str">
-        <x:v>https://doi.org/10.1016/j.image.2022.116891</x:v>
-      </x:c>
-      <x:c r="F41" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" t="str">
-        <x:v>Exploring the Advantages of Quantum Generative Adversarial Networks in Generative Chemistry</x:v>
-      </x:c>
-      <x:c r="B42" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C42" t="str">
-        <x:v>Journal of Chemical Information and Modeling</x:v>
-      </x:c>
-      <x:c r="D42" t="str">
-        <x:v>Po-Yu Kao,Ya-Chu Yang,Wei-Yin Chiang,Jen-Yueh Hsiao,Yudong Cao,Alex Aliper,Feng Ren,Alán Aspuru-Guzik,Alex Zhavoronkov,Min-Hsiu Hsieh,Yen-Chu Lin</x:v>
-      </x:c>
-      <x:c r="E42" t="str">
-        <x:v>https://doi.org/10.1021/acs.jcim.3c00562</x:v>
-      </x:c>
-      <x:c r="F42" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" t="str">
-        <x:v>A Survey of Recent Advances in Quantum Generative Adversarial Networks</x:v>
-      </x:c>
-      <x:c r="B43" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C43" t="str">
-        <x:v>MDPI</x:v>
-      </x:c>
-      <x:c r="D43" t="str">
-        <x:v> Tuan A. Ngo,bTuyen Nguyen, Truong Cong Thang</x:v>
-      </x:c>
-      <x:c r="E43" t="str">
-        <x:v>https://doi.org/10.3390/electronics12040856</x:v>
-      </x:c>
-      <x:c r="F43" t="str">
-        <x:v>QGenerative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" t="str">
-        <x:v>Hybrid Quantum–Classical Generative Adversarial Network for High-Resolution Image Generation</x:v>
-      </x:c>
-      <x:c r="B44" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C44" t="str">
-        <x:v>IEEE</x:v>
-      </x:c>
-      <x:c r="D44" t="str">
-        <x:v>Shu Lok Tsang; Maxwell T. West; Sarah M. Erfani; Muhammad Usman</x:v>
-      </x:c>
-      <x:c r="E44" t="str">
-        <x:v>https://doi.org/10.1109/TQE.2023.3319319</x:v>
       </x:c>
       <x:c r="F44" t="str">
         <x:v>QGenerative</x:v>
@@ -1217,19 +1217,19 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="str">
-        <x:v>MosaiQ: Quantum Generative Adversarial Networks for Image Generation on NISQ Computers</x:v>
+        <x:v>Investigating Training Dynamics of Quantum Generative Adversarial Networks</x:v>
       </x:c>
       <x:c r="B45" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>Bulletin of the American Physical Society </x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>Daniel Silver, Tirthak Patel, William Cutler, Aditya Ranjan, Harshitta Gandhi, Devesh Tiwari</x:v>
+        <x:v>Rajapakse, Renuka, and McCord Murray.</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.2308.11096</x:v>
+        <x:v>https://meetings.aps.org/Meeting/DAMOP24/Session/R11.1</x:v>
       </x:c>
       <x:c r="F45" t="str">
         <x:v>QGenerative</x:v>
@@ -1237,19 +1237,19 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="str">
-        <x:v>Variational measurement-based quantum computation for generative modeling</x:v>
+        <x:v>Latent Style-based Quantum GAN for high-quality Image Generation</x:v>
       </x:c>
       <x:c r="B46" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C46" t="str">
         <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D46" t="str">
-        <x:v>Arunava Majumder, Marius Krumm, Tina Radkohl, Hendrik Poulsen Nautrup, Sofiene Jerbi, Hans J. Briegel</x:v>
+        <x:v>Chang, Su Yeon, et al.</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.2310.13524</x:v>
+        <x:v>https://arxiv.org/pdf/2406.02668</x:v>
       </x:c>
       <x:c r="F46" t="str">
         <x:v>QGenerative</x:v>
@@ -1257,19 +1257,19 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="str">
-        <x:v>IQGAN: Robust Quantum Generative Adversarial Network for Image Synthesis On NISQ Devices</x:v>
+        <x:v>Recent Advances for Quantum Neural Networks in Generative Learning</x:v>
       </x:c>
       <x:c r="B47" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>IEEE</x:v>
+        <x:v> IEEE Transactions on Pattern Analysis and Machine Intelligence</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>Cheng Chu; Grant Skipper; Martin Swany; Fan Chen</x:v>
+        <x:v>Jinkai Tian, Xiaoyu Sun, Yuxuan Du, Shanshan Zhao, Qing Liu, Kaining Zhang, Wei Yi, Wanrong Huang, Chaoyue Wang, Xingyao Wu, Min-Hsiu Hsieh, Tongliang Liu, Wenjing Yang, Dacheng Tao</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>https://doi.org/10.1109/ICASSP49357.2023.10096772</x:v>
+        <x:v>https://doi.org/10.1109/TPAMI.2023.3272029</x:v>
       </x:c>
       <x:c r="F47" t="str">
         <x:v>QGenerative</x:v>
@@ -1277,19 +1277,19 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" t="str">
-        <x:v>Quantum generative adversarial learning in photonics</x:v>
+        <x:v>Hybrid quantum–classical generative adversarial networks for image generation via learning discrete distribution</x:v>
       </x:c>
       <x:c r="B48" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>OPTICA PUBLISHING GROUP</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>Yizhi Wang, Shichuan Xue, Yaxuan Wang, Yong Liu, Jiangfang Ding, Weixu Shi, Dongyang Wang, Yingwen Liu, Xiang Fu, Guangyao Huang, Anqi Huang, Mingtang Deng, and Junjie Wu</x:v>
+        <x:v>Nan-Run Zhou,  Tian-Feng Zhang,  Xin-Wen Xie,  Jun-Yun Wu</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>https://opg.optica.org/ol/abstract.cfm?URI=ol-48-20-5197</x:v>
+        <x:v>https://doi.org/10.1016/j.image.2022.116891</x:v>
       </x:c>
       <x:c r="F48" t="str">
         <x:v>QGenerative</x:v>
@@ -1297,19 +1297,19 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="str">
-        <x:v>Quantum conditional generative adversarial network based on patch method for abnormal electrocardiogram generation</x:v>
+        <x:v>Exploring the Advantages of Quantum Generative Adversarial Networks in Generative Chemistry</x:v>
       </x:c>
       <x:c r="B49" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>Journal of Chemical Information and Modeling</x:v>
       </x:c>
       <x:c r="D49" t="str">
-        <x:v>Zhiguo Qu, Wenke Shi, Prayag Tiwari</x:v>
+        <x:v>Po-Yu Kao,Ya-Chu Yang,Wei-Yin Chiang,Jen-Yueh Hsiao,Yudong Cao,Alex Aliper,Feng Ren,Alán Aspuru-Guzik,Alex Zhavoronkov,Min-Hsiu Hsieh,Yen-Chu Lin</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>https://doi.org/10.1016/j.compbiomed.2023.107549</x:v>
+        <x:v>https://doi.org/10.1021/acs.jcim.3c00562</x:v>
       </x:c>
       <x:c r="F49" t="str">
         <x:v>QGenerative</x:v>
@@ -1317,19 +1317,19 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" t="str">
-        <x:v>Introducing nonlinear activations into quantum generative models</x:v>
+        <x:v>A Survey of Recent Advances in Quantum Generative Adversarial Networks</x:v>
       </x:c>
       <x:c r="B50" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>ASP</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>Kaitlin Gili, Mykolas Sveistrys, and Chris Balance</x:v>
+        <x:v> Tuan A. Ngo,bTuyen Nguyen, Truong Cong Thang</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevA.107.012406</x:v>
+        <x:v>https://doi.org/10.3390/electronics12040856</x:v>
       </x:c>
       <x:c r="F50" t="str">
         <x:v>QGenerative</x:v>
@@ -1337,19 +1337,19 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="str">
-        <x:v>Trainability barriers and opportunities in quantum generative modeling</x:v>
+        <x:v>Hybrid Quantum–Classical Generative Adversarial Network for High-Resolution Image Generation</x:v>
       </x:c>
       <x:c r="B51" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>Manuel S. Rudolph, Sacha Lerch, Supanut Thanasilp, Oriel Kiss, Sofia Vallecorsa, Michele Grossi, Zoë Holmes</x:v>
+        <x:v>Shu Lok Tsang; Maxwell T. West; Sarah M. Erfani; Muhammad Usman</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.2305.02881</x:v>
+        <x:v>https://doi.org/10.1109/TQE.2023.3319319</x:v>
       </x:c>
       <x:c r="F51" t="str">
         <x:v>QGenerative</x:v>
@@ -1357,19 +1357,19 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" t="str">
-        <x:v>Towards a scalable discrete quantum generative adversarial neural network</x:v>
+        <x:v>MosaiQ: Quantum Generative Adversarial Networks for Image Generation on NISQ Computers</x:v>
       </x:c>
       <x:c r="B52" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>IOPSCIENCE</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>Smit Chaudhary, Patrick Huembeli, Ian MacCormack, Taylor L Patti, Jean Kossaifi and Alexey Galda</x:v>
+        <x:v>Daniel Silver, Tirthak Patel, William Cutler, Aditya Ranjan, Harshitta Gandhi, Devesh Tiwari</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>https://doi.org/10.1088/2058-9565/acc4e4</x:v>
+        <x:v>https://doi.org/10.48550/arXiv.2308.11096</x:v>
       </x:c>
       <x:c r="F52" t="str">
         <x:v>QGenerative</x:v>
@@ -1377,50 +1377,197 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="str">
-        <x:v>Q-Flow: Generative Modeling for Differential Equations of Open Quantum Dynamics with Normalizing Flows</x:v>
+        <x:v>Variational measurement-based quantum computation for generative modeling</x:v>
       </x:c>
       <x:c r="B53" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C53" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>Arunava Majumder, Marius Krumm, Tina Radkohl, Hendrik Poulsen Nautrup, Sofiene Jerbi, Hans J. Briegel</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>https://doi.org/10.48550/arXiv.2310.13524</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>IQGAN: Robust Quantum Generative Adversarial Network for Image Synthesis On NISQ Devices</x:v>
+      </x:c>
+      <x:c r="B54" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>IEEE</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>Cheng Chu; Grant Skipper; Martin Swany; Fan Chen</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>https://doi.org/10.1109/ICASSP49357.2023.10096772</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>Quantum generative adversarial learning in photonics</x:v>
+      </x:c>
+      <x:c r="B55" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>OPTICA PUBLISHING GROUP</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>Yizhi Wang, Shichuan Xue, Yaxuan Wang, Yong Liu, Jiangfang Ding, Weixu Shi, Dongyang Wang, Yingwen Liu, Xiang Fu, Guangyao Huang, Anqi Huang, Mingtang Deng, and Junjie Wu</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>https://opg.optica.org/ol/abstract.cfm?URI=ol-48-20-5197</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>Quantum conditional generative adversarial network based on patch method for abnormal electrocardiogram generation</x:v>
+      </x:c>
+      <x:c r="B56" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>ScienceDirect</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>Zhiguo Qu, Wenke Shi, Prayag Tiwari</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>https://doi.org/10.1016/j.compbiomed.2023.107549</x:v>
+      </x:c>
+      <x:c r="F56" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>Introducing nonlinear activations into quantum generative models</x:v>
+      </x:c>
+      <x:c r="B57" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>ASP</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>Kaitlin Gili, Mykolas Sveistrys, and Chris Balance</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>https://doi.org/10.1103/PhysRevA.107.012406</x:v>
+      </x:c>
+      <x:c r="F57" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>Trainability barriers and opportunities in quantum generative modeling</x:v>
+      </x:c>
+      <x:c r="B58" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>Manuel S. Rudolph, Sacha Lerch, Supanut Thanasilp, Oriel Kiss, Sofia Vallecorsa, Michele Grossi, Zoë Holmes</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>https://doi.org/10.48550/arXiv.2305.02881</x:v>
+      </x:c>
+      <x:c r="F58" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>Towards a scalable discrete quantum generative adversarial neural network</x:v>
+      </x:c>
+      <x:c r="B59" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>IOPSCIENCE</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>Smit Chaudhary, Patrick Huembeli, Ian MacCormack, Taylor L Patti, Jean Kossaifi and Alexey Galda</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>https://doi.org/10.1088/2058-9565/acc4e4</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>QGenerative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>Q-Flow: Generative Modeling for Differential Equations of Open Quantum Dynamics with Normalizing Flows</x:v>
+      </x:c>
+      <x:c r="B60" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
         <x:v>PMLR</x:v>
       </x:c>
-      <x:c r="D53" t="str">
+      <x:c r="D60" t="str">
         <x:v>Owen M Dugan, Peter Y. Lu, Rumen Dangovski, Di Luo, Marin Soljacic</x:v>
       </x:c>
-      <x:c r="E53" t="str">
+      <x:c r="E60" t="str">
         <x:v>https://proceedings.mlr.press/v202/dugan23a.html</x:v>
       </x:c>
-      <x:c r="F53" t="str">
+      <x:c r="F60" t="str">
         <x:v>QGenerative</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="R1936eb535c1c46fb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="R8bfe9cd62c754159"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="Rfdff6b289ecf46cb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="R7416826e7dbc4eb8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R62bc6308710e47c7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R19a614fdf7f4429b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R957c4a2cab004b6c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R3204ae40e9bb4865"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="R972879cd3baf4fdc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="R70f8fb8beb9e424c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R05ae5b0b19ef4ab5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Ra2fdae9ae4f84100"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="R70ecd9255d5d4b2d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="Rb9ecb13331754bf5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Rd4ff558a889d4fc4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="Rc12acc3caf824e27"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R2c6dd474409e47e5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="Rca9eea896e4e4699"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="Rd593a91212824e57"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="Rbc7c7ea4da1c4e5a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R30cfe16b91974f8f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="R75212cd77c1b4ed9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R02c820d862af4ac2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R3bc2f2ac3a2f43d4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="R35a8c6a44aef4d85"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="Rca7f55225e9149db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="R2aedf8b00aab407e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="Rc4ab6fea13e0411c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R6559df3f81064519"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="Rd6fd3340dcc24a08"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="Raa88e2d7b03b4a2f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R46d4561f41404014"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="R031cb9438e484630"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="R397ce7aa52df48a2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rdd538832d03b4f32"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R9ca437d5fda74eab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="Rf8e97da443e14b60"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="R61f16b4984f040d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="R8b51fa30461843d7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R46064e0d33a4456c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="Ra34b6d6093674da4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="Rd6cd014462b643ec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R10b0257a2d794cdb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="Rd79ffc49d3d643d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R1e98da2ff30c48ec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="R5b72dec8b240467c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R5c83894d924e4c6e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R33af12cc87954682"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R880bb02333ce4faa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="Rda4e52c2c7bf4c7d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="R54f454bc25094f01"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="R01a0e032081141d9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R398779fcd01a4e52"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="Rddfed7e0ac5747bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R343da3f4f6154f03"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>